<commit_message>
feat: Ban Mong - thiet bi bu muc nuoc (tu cang + khoa bao), do nhay theo khao sat
- mooringEquilibrium: che do 'device' (day luc cang khong doi, hanh trinh +-S);
  doi trong treo mot minh khong giu duoc be: troi het hanh trinh, luc day gap 1,2-2,8 lan
- catalogue luu lockFailure; canh bao dau tien neu so khi khoa hong
- bang neo muc VI: yeu cau ky thuat bo tu cang va bo khoa fail-safe
- scripts/sensitivityBanMong.ts: do nhay theo cu dat bo / bun day, cao do neo, EA
- test tay cho che do device

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/docs_ban_mong/HOBANMONG_THONG_KE_VAT_TU_NEO.xlsx
+++ b/public/docs_ban_mong/HOBANMONG_THONG_KE_VAT_TU_NEO.xlsx
@@ -1071,7 +1071,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>50</row>
+      <row>51</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1490133" cy="1117600"/>
@@ -1096,7 +1096,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>51</row>
+      <row>52</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1490133" cy="1117600"/>
@@ -1121,7 +1121,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>52</row>
+      <row>53</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1490133" cy="1117600"/>
@@ -1146,7 +1146,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>53</row>
+      <row>54</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1490133" cy="1117600"/>
@@ -1171,7 +1171,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>55</row>
+      <row>56</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1490133" cy="1117600"/>
@@ -1196,7 +1196,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>56</row>
+      <row>57</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="1490133" cy="1117600"/>
@@ -1546,7 +1546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I59"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6.8" customWidth="1" min="1" max="1"/>
@@ -3109,7 +3109,7 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>THIẾT BỊ BÙ DAO ĐỘNG MỰC NƯỚC (BẮT BUỘC, CHƯA THIẾT KẾ — KHÔNG ĐẶT HÀNG THEO MỤC NÀY)</t>
+          <t>THIẾT BỊ BÙ DAO ĐỘNG MỰC NƯỚC (BẮT BUỘC — CHỈ MỚI CÓ YÊU CẦU KỸ THUẬT, CHƯA CHỌN LOẠI: KHÔNG ĐẶT HÀNG THEO MỤC NÀY)</t>
         </is>
       </c>
       <c r="C48" s="4" t="n"/>
@@ -3126,7 +3126,7 @@
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>Thiết bị bù dao động mực nước mỗi dây</t>
+          <t>Bộ tự căng / thu xả cáp mỗi dây (đối trọng hoặc tời)</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
@@ -3136,7 +3136,7 @@
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>Đối trọng treo / bộ tự căng giữ dây vừa căng ở mọi mực nước (649,50–669,05 m); hành trình thu–xả: dây đáy tới 15,9 m, dây bờ tới 4,6 m; phải KHÓA được khi bão</t>
+          <t>Giữ lực căng đặt 5 kN ở mọi mực nước 649,50–669,05 m; hành trình thu–xả: dây đáy 15,9 m, dây bờ 4,6 m, cộng 3 m dư mỗi chiều</t>
         </is>
       </c>
       <c r="E49" s="6" t="inlineStr">
@@ -3149,7 +3149,7 @@
       </c>
       <c r="G49" s="6" t="inlineStr">
         <is>
-          <t>CHƯA thiết kế</t>
+          <t>CHƯA chọn loại</t>
         </is>
       </c>
       <c r="H49" s="9" t="n">
@@ -3157,65 +3157,69 @@
       </c>
       <c r="I49" s="7" t="inlineStr">
         <is>
-          <t>Lực dây 54,9–107,0 kN của engine CHỈ đúng khi có thiết bị này (cáp cắt cố định thì không cáp PES nào đủ — bảng so sánh ở Mục 4 trên web). Pre-FS gợi ý phao chỉ hướng ~2,5 t</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="31" customHeight="1">
-      <c r="A50" s="4" t="inlineStr">
+          <t>Yêu cầu của mô hình cân bằng (mooringEquilibrium.ts): dây luôn vừa căng ở mọi mực nước. Đối trọng treo một mình KHÔNG giữ được bè: nếu không khóa, bè trôi 5,1–6,3 m hết hành trình dư rồi lực dây vọt tới 108–296 kN</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="46" customHeight="1">
+      <c r="A50" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>Bộ khóa / phanh cáp chống bão mỗi dây (fail-safe)</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>(chưa có hình)</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>Khóa cáp khi gió vượt ngưỡng, giữ tới lực đứt của cáp chính (PES-28: 235 kN; PES-32: 305 kN; PES-36: 385 kN) để khóa không yếu hơn cáp; mất điện / mất tín hiệu thì tự khóa (lò xo ép phanh)</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="inlineStr">
+        <is>
+          <t>bộ</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="n">
+        <v>271</v>
+      </c>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>CHƯA chọn loại</t>
+        </is>
+      </c>
+      <c r="H50" s="9" t="n">
+        <v>271</v>
+      </c>
+      <c r="I50" s="7" t="inlineStr">
+        <is>
+          <t>Lực dây, đế, cọc của bảng này chỉ đúng khi khóa làm việc. Cần: tín hiệu gió + dự phòng, kiểm tra định kỳ, thử tải; khóa hỏng thì hệ số an toàn cáp chỉ còn 1,3–2,8 (xem cảnh báo ở Header). Pre-FS gợi ý phao chỉ hướng ~2,5 t — chưa đánh giá</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="31" customHeight="1">
+      <c r="A51" s="4" t="inlineStr">
         <is>
           <t>VII</t>
         </is>
       </c>
-      <c r="B50" s="5" t="inlineStr">
+      <c r="B51" s="5" t="inlineStr">
         <is>
           <t>TỔNG THÉP HỆ NEO (chi tiết theo đường kính: sheet TongHop_Thep)</t>
         </is>
       </c>
-      <c r="C50" s="4" t="n"/>
-      <c r="D50" s="5" t="n"/>
-      <c r="E50" s="4" t="n"/>
-      <c r="F50" s="5" t="n"/>
-      <c r="G50" s="4" t="n"/>
-      <c r="H50" s="5" t="n"/>
-      <c r="I50" s="5" t="n"/>
-    </row>
-    <row r="51" ht="92" customHeight="1">
-      <c r="A51" s="6" t="n">
-        <v>39</v>
-      </c>
-      <c r="B51" s="7" t="inlineStr">
-        <is>
-          <t>Thép chủ cọc Φ25</t>
-        </is>
-      </c>
-      <c r="C51" s="6" t="n"/>
-      <c r="D51" s="7" t="inlineStr">
-        <is>
-          <t>CB400-V, thanh vằn</t>
-        </is>
-      </c>
-      <c r="E51" s="6" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="F51" s="9" t="n">
-        <v>27009</v>
-      </c>
-      <c r="G51" s="6" t="inlineStr">
-        <is>
-          <t>3%</t>
-        </is>
-      </c>
-      <c r="H51" s="9" t="n">
-        <v>27820</v>
-      </c>
-      <c r="I51" s="7" t="inlineStr">
-        <is>
-          <t>Lồng thép cọc khoan nhồi (engine)</t>
-        </is>
-      </c>
+      <c r="C51" s="4" t="n"/>
+      <c r="D51" s="5" t="n"/>
+      <c r="E51" s="4" t="n"/>
+      <c r="F51" s="5" t="n"/>
+      <c r="G51" s="4" t="n"/>
+      <c r="H51" s="5" t="n"/>
+      <c r="I51" s="5" t="n"/>
     </row>
     <row r="52" ht="92" customHeight="1">
       <c r="A52" s="6" t="n">
@@ -3223,7 +3227,7 @@
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>Thép chủ cọc Φ28</t>
+          <t>Thép chủ cọc Φ25</t>
         </is>
       </c>
       <c r="C52" s="6" t="n"/>
@@ -3238,7 +3242,7 @@
         </is>
       </c>
       <c r="F52" s="9" t="n">
-        <v>8231</v>
+        <v>27009</v>
       </c>
       <c r="G52" s="6" t="inlineStr">
         <is>
@@ -3246,7 +3250,7 @@
         </is>
       </c>
       <c r="H52" s="9" t="n">
-        <v>8478</v>
+        <v>27820</v>
       </c>
       <c r="I52" s="7" t="inlineStr">
         <is>
@@ -3260,13 +3264,13 @@
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>Thép đai xoắn Φ8</t>
+          <t>Thép chủ cọc Φ28</t>
         </is>
       </c>
       <c r="C53" s="6" t="n"/>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>CB240-T, thép cuộn</t>
+          <t>CB400-V, thanh vằn</t>
         </is>
       </c>
       <c r="E53" s="6" t="inlineStr">
@@ -3275,19 +3279,19 @@
         </is>
       </c>
       <c r="F53" s="9" t="n">
-        <v>3563</v>
+        <v>8231</v>
       </c>
       <c r="G53" s="6" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>3%</t>
         </is>
       </c>
       <c r="H53" s="9" t="n">
-        <v>3742</v>
+        <v>8478</v>
       </c>
       <c r="I53" s="7" t="inlineStr">
         <is>
-          <t>Cọc khoan nhồi (engine)</t>
+          <t>Lồng thép cọc khoan nhồi (engine)</t>
         </is>
       </c>
     </row>
@@ -3297,13 +3301,13 @@
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>Thép bản đế Φ12</t>
+          <t>Thép đai xoắn Φ8</t>
         </is>
       </c>
       <c r="C54" s="6" t="n"/>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>CB400-V (lưới đế)</t>
+          <t>CB240-T, thép cuộn</t>
         </is>
       </c>
       <c r="E54" s="6" t="inlineStr">
@@ -3312,39 +3316,35 @@
         </is>
       </c>
       <c r="F54" s="9" t="n">
-        <v>17935</v>
+        <v>3563</v>
       </c>
       <c r="G54" s="6" t="inlineStr">
         <is>
-          <t>3%</t>
+          <t>5%</t>
         </is>
       </c>
       <c r="H54" s="9" t="n">
-        <v>18474</v>
+        <v>3742</v>
       </c>
       <c r="I54" s="7" t="inlineStr">
         <is>
-          <t>Đế BTCT (engine)</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="46" customHeight="1">
+          <t>Cọc khoan nhồi (engine)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="92" customHeight="1">
       <c r="A55" s="6" t="n">
         <v>43</v>
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>Thép ống vít Ø89×5</t>
-        </is>
-      </c>
-      <c r="C55" s="6" t="inlineStr">
-        <is>
-          <t>(chưa có hình)</t>
-        </is>
-      </c>
+          <t>Thép bản đế Φ12</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="n"/>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>Ống thép mạ kẽm nhúng nóng</t>
+          <t>CB400-V (lưới đế)</t>
         </is>
       </c>
       <c r="E55" s="6" t="inlineStr">
@@ -3353,35 +3353,39 @@
         </is>
       </c>
       <c r="F55" s="9" t="n">
-        <v>15599</v>
+        <v>17935</v>
       </c>
       <c r="G55" s="6" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>3%</t>
         </is>
       </c>
       <c r="H55" s="9" t="n">
-        <v>16379</v>
+        <v>18474</v>
       </c>
       <c r="I55" s="7" t="inlineStr">
         <is>
-          <t>10,36 kg/m</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="92" customHeight="1">
+          <t>Đế BTCT (engine)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="46" customHeight="1">
       <c r="A56" s="6" t="n">
         <v>44</v>
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>Thép tấm bản mã + tai neo (đầu cọc, đài, đế)</t>
-        </is>
-      </c>
-      <c r="C56" s="6" t="n"/>
+          <t>Thép ống vít Ø89×5</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>(chưa có hình)</t>
+        </is>
+      </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>SS400 mạ kẽm nhúng nóng</t>
+          <t>Ống thép mạ kẽm nhúng nóng</t>
         </is>
       </c>
       <c r="E56" s="6" t="inlineStr">
@@ -3390,7 +3394,7 @@
         </is>
       </c>
       <c r="F56" s="9" t="n">
-        <v>8248</v>
+        <v>15599</v>
       </c>
       <c r="G56" s="6" t="inlineStr">
         <is>
@@ -3398,11 +3402,11 @@
         </is>
       </c>
       <c r="H56" s="9" t="n">
-        <v>8661</v>
+        <v>16379</v>
       </c>
       <c r="I56" s="7" t="inlineStr">
         <is>
-          <t>271 bộ</t>
+          <t>10,36 kg/m</t>
         </is>
       </c>
     </row>
@@ -3412,13 +3416,13 @@
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>Thép neo bản mã Φ22</t>
+          <t>Thép tấm bản mã + tai neo (đầu cọc, đài, đế)</t>
         </is>
       </c>
       <c r="C57" s="6" t="n"/>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>CB400-V</t>
+          <t>SS400 mạ kẽm nhúng nóng</t>
         </is>
       </c>
       <c r="E57" s="6" t="inlineStr">
@@ -3427,39 +3431,35 @@
         </is>
       </c>
       <c r="F57" s="9" t="n">
-        <v>1582</v>
+        <v>8248</v>
       </c>
       <c r="G57" s="6" t="inlineStr">
         <is>
-          <t>3%</t>
+          <t>5%</t>
         </is>
       </c>
       <c r="H57" s="9" t="n">
-        <v>1629</v>
+        <v>8661</v>
       </c>
       <c r="I57" s="7" t="inlineStr">
         <is>
-          <t>271 bộ × 4 thanh</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="46" customHeight="1">
+          <t>271 bộ</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="92" customHeight="1">
       <c r="A58" s="6" t="n">
         <v>46</v>
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>Thép đài cọc đôi</t>
-        </is>
-      </c>
-      <c r="C58" s="6" t="inlineStr">
-        <is>
-          <t>(chưa có hình)</t>
-        </is>
-      </c>
+          <t>Thép neo bản mã Φ22</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="n"/>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>CB400-V Φ16, Φ12; CB240-T Φ10</t>
+          <t>CB400-V</t>
         </is>
       </c>
       <c r="E58" s="6" t="inlineStr">
@@ -3468,19 +3468,19 @@
         </is>
       </c>
       <c r="F58" s="9" t="n">
-        <v>3288</v>
+        <v>1582</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>3%</t>
         </is>
       </c>
       <c r="H58" s="9" t="n">
-        <v>3453</v>
+        <v>1629</v>
       </c>
       <c r="I58" s="7" t="inlineStr">
         <is>
-          <t>twinPileCap.ts</t>
+          <t>271 bộ × 4 thanh</t>
         </is>
       </c>
     </row>
@@ -3490,36 +3490,77 @@
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
+          <t>Thép đài cọc đôi</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>(chưa có hình)</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>CB400-V Φ16, Φ12; CB240-T Φ10</t>
+        </is>
+      </c>
+      <c r="E59" s="6" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="F59" s="9" t="n">
+        <v>3288</v>
+      </c>
+      <c r="G59" s="6" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="H59" s="9" t="n">
+        <v>3453</v>
+      </c>
+      <c r="I59" s="7" t="inlineStr">
+        <is>
+          <t>twinPileCap.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="46" customHeight="1">
+      <c r="A60" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="B60" s="7" t="inlineStr">
+        <is>
           <t>TỔNG THÉP HỆ NEO</t>
         </is>
       </c>
-      <c r="C59" s="6" t="inlineStr">
+      <c r="C60" s="6" t="inlineStr">
         <is>
           <t>(chưa có hình)</t>
         </is>
       </c>
-      <c r="D59" s="7" t="inlineStr">
+      <c r="D60" s="7" t="inlineStr">
         <is>
           <t>Thép thanh + thép ống vít + thép tấm bản nắp</t>
         </is>
       </c>
-      <c r="E59" s="6" t="inlineStr">
+      <c r="E60" s="6" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="F59" s="9" t="n">
+      <c r="F60" s="9" t="n">
         <v>85455</v>
       </c>
-      <c r="G59" s="6" t="inlineStr">
+      <c r="G60" s="6" t="inlineStr">
         <is>
           <t>theo từng loại</t>
         </is>
       </c>
-      <c r="H59" s="9" t="n">
+      <c r="H60" s="9" t="n">
         <v>88636</v>
       </c>
-      <c r="I59" s="7" t="inlineStr">
+      <c r="I60" s="7" t="inlineStr">
         <is>
           <t>Chưa gồm nắp khóa vít, tấm chia (chưa có kích thước chi tiết)</t>
         </is>

</xml_diff>

<commit_message>
feat: Huoi Vanh - tinh lai luc day can bang theo muc nuoc (23/10/2026)
- Luc day Huoi Vanh theo mo hinh can bang tinh (nhu Ban Mong), cao trinh 380/384.5/386;
  chinh day moi 1 m muc nuoc la dieu kien bat buoc; day < 4 m la day du phong
- T 64-150 kN, cap PES-28..40, 262 coc D350 (coc doi BE 3A), 32 de 84.7 m3
- Bang thong ke vat tu neo: thiet ke so bo dau coc / dai coc doi / tai neo de cho ca Huoi Vanh,
  doan xich chinh theo hanh trinh that; them bang vat tu be pin vao tai lieu dinh kem
- Thuyet minh, bang tinh, ban ve neo, ban ve coc ven bo sinh lai; tai lieu ghi ngay tinh lai

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/docs_ban_mong/HOBANMONG_THONG_KE_VAT_TU_NEO.xlsx
+++ b/public/docs_ban_mong/HOBANMONG_THONG_KE_VAT_TU_NEO.xlsx
@@ -3891,7 +3891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O12"/>
+  <dimension ref="A1:P12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.83203125" customWidth="1" min="1" max="1"/>
@@ -3904,11 +3904,12 @@
     <col width="14.83203125" customWidth="1" min="8" max="8"/>
     <col width="14.83203125" customWidth="1" min="9" max="9"/>
     <col width="14.83203125" customWidth="1" min="10" max="10"/>
-    <col width="12.83203125" customWidth="1" min="11" max="11"/>
+    <col width="14.83203125" customWidth="1" min="11" max="11"/>
     <col width="12.83203125" customWidth="1" min="12" max="12"/>
-    <col width="9.83203125" customWidth="1" min="13" max="13"/>
+    <col width="12.83203125" customWidth="1" min="13" max="13"/>
     <col width="9.83203125" customWidth="1" min="14" max="14"/>
     <col width="9.83203125" customWidth="1" min="15" max="15"/>
+    <col width="9.83203125" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3921,7 +3922,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Mỗi cọc: D350 đổ tại chỗ, lồng thép theo bè, đai xoắn Φ8 a150 CB240-T, mũ cọc + bản nắp 400×400×20 + tai neo + 4Φ25 L600 ngàm bản nắp.</t>
+          <t>Mỗi cọc: D350 đổ tại chỗ, lồng thép theo bè, đai xoắn Φ8 a150 CB240-T. Mỗi điểm neo một đầu cọc (bản mã + tai neo + thép neo, shorePileHead.ts) hoặc, ở điểm cọc đôi, một đài BTCT nối hai đầu cọc (twinPileCap.ts).</t>
         </is>
       </c>
     </row>
@@ -3973,30 +3974,35 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>Râu thép 4Φ25 L600 (kg)</t>
+          <t>Thép neo bản mã (kg)</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Bản nắp SS400 (kg)</t>
+          <t>Bản mã + tai neo SS400 (kg)</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
+          <t>Thép đài cọc đôi (kg)</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
           <t>Tổng thép (kg)</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>T dây (kN)</t>
         </is>
       </c>
-      <c r="N3" s="3" t="inlineStr">
+      <c r="O3" s="3" t="inlineStr">
         <is>
           <t>BP-1 ngang</t>
         </is>
       </c>
-      <c r="O3" s="3" t="inlineStr">
+      <c r="P3" s="3" t="inlineStr">
         <is>
           <t>BP-2 uốn</t>
         </is>
@@ -4035,21 +4041,24 @@
         <v>615</v>
       </c>
       <c r="J4" s="11" t="n">
-        <v>351</v>
+        <v>136</v>
       </c>
       <c r="K4" s="11" t="n">
-        <v>955</v>
+        <v>559</v>
       </c>
       <c r="L4" s="11" t="n">
-        <v>7720</v>
+        <v>718</v>
       </c>
       <c r="M4" s="11" t="n">
+        <v>7827</v>
+      </c>
+      <c r="N4" s="11" t="n">
         <v>104.9</v>
       </c>
-      <c r="N4" s="11" t="n">
+      <c r="O4" s="11" t="n">
         <v>0.5</v>
       </c>
-      <c r="O4" s="11" t="n">
+      <c r="P4" s="11" t="n">
         <v>0.8100000000000001</v>
       </c>
     </row>
@@ -4086,21 +4095,24 @@
         <v>405</v>
       </c>
       <c r="J5" s="11" t="n">
-        <v>231</v>
+        <v>179</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>628</v>
+        <v>736</v>
       </c>
       <c r="L5" s="11" t="n">
-        <v>6049</v>
+        <v>0</v>
       </c>
       <c r="M5" s="11" t="n">
+        <v>6105</v>
+      </c>
+      <c r="N5" s="11" t="n">
         <v>73.7</v>
       </c>
-      <c r="N5" s="11" t="n">
+      <c r="O5" s="11" t="n">
         <v>0.64</v>
       </c>
-      <c r="O5" s="11" t="n">
+      <c r="P5" s="11" t="n">
         <v>0.87</v>
       </c>
     </row>
@@ -4137,21 +4149,24 @@
         <v>551</v>
       </c>
       <c r="J6" s="11" t="n">
-        <v>314</v>
+        <v>122</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>854</v>
+        <v>500</v>
       </c>
       <c r="L6" s="11" t="n">
-        <v>6907</v>
+        <v>642</v>
       </c>
       <c r="M6" s="11" t="n">
+        <v>7003</v>
+      </c>
+      <c r="N6" s="11" t="n">
         <v>106.9</v>
       </c>
-      <c r="N6" s="11" t="n">
+      <c r="O6" s="11" t="n">
         <v>0.51</v>
       </c>
-      <c r="O6" s="11" t="n">
+      <c r="P6" s="11" t="n">
         <v>0.82</v>
       </c>
     </row>
@@ -4188,21 +4203,24 @@
         <v>518</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>296</v>
+        <v>115</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>804</v>
+        <v>471</v>
       </c>
       <c r="L7" s="11" t="n">
-        <v>6501</v>
+        <v>605</v>
       </c>
       <c r="M7" s="11" t="n">
+        <v>6591</v>
+      </c>
+      <c r="N7" s="11" t="n">
         <v>94.59999999999999</v>
       </c>
-      <c r="N7" s="11" t="n">
+      <c r="O7" s="11" t="n">
         <v>0.45</v>
       </c>
-      <c r="O7" s="11" t="n">
+      <c r="P7" s="11" t="n">
         <v>0.71</v>
       </c>
     </row>
@@ -4239,21 +4257,24 @@
         <v>292</v>
       </c>
       <c r="J8" s="11" t="n">
-        <v>166</v>
+        <v>129</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>452</v>
+        <v>530</v>
       </c>
       <c r="L8" s="11" t="n">
-        <v>4356</v>
+        <v>0</v>
       </c>
       <c r="M8" s="11" t="n">
+        <v>4396</v>
+      </c>
+      <c r="N8" s="11" t="n">
         <v>75</v>
       </c>
-      <c r="N8" s="11" t="n">
+      <c r="O8" s="11" t="n">
         <v>0.65</v>
       </c>
-      <c r="O8" s="11" t="n">
+      <c r="P8" s="11" t="n">
         <v>0.89</v>
       </c>
     </row>
@@ -4290,21 +4311,24 @@
         <v>49</v>
       </c>
       <c r="J9" s="11" t="n">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="L9" s="11" t="n">
-        <v>609</v>
+        <v>0</v>
       </c>
       <c r="M9" s="11" t="n">
+        <v>616</v>
+      </c>
+      <c r="N9" s="11" t="n">
         <v>54.9</v>
       </c>
-      <c r="N9" s="11" t="n">
+      <c r="O9" s="11" t="n">
         <v>0.47</v>
       </c>
-      <c r="O9" s="11" t="n">
+      <c r="P9" s="11" t="n">
         <v>0.75</v>
       </c>
     </row>
@@ -4341,21 +4365,24 @@
         <v>648</v>
       </c>
       <c r="J10" s="11" t="n">
-        <v>370</v>
+        <v>143</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>1005</v>
+        <v>589</v>
       </c>
       <c r="L10" s="11" t="n">
-        <v>8126</v>
+        <v>756</v>
       </c>
       <c r="M10" s="11" t="n">
+        <v>8239</v>
+      </c>
+      <c r="N10" s="11" t="n">
         <v>107</v>
       </c>
-      <c r="N10" s="11" t="n">
+      <c r="O10" s="11" t="n">
         <v>0.51</v>
       </c>
-      <c r="O10" s="11" t="n">
+      <c r="P10" s="11" t="n">
         <v>0.82</v>
       </c>
     </row>
@@ -4392,21 +4419,24 @@
         <v>486</v>
       </c>
       <c r="J11" s="11" t="n">
-        <v>277</v>
+        <v>107</v>
       </c>
       <c r="K11" s="11" t="n">
-        <v>754</v>
+        <v>442</v>
       </c>
       <c r="L11" s="11" t="n">
-        <v>6095</v>
+        <v>567</v>
       </c>
       <c r="M11" s="11" t="n">
+        <v>6180</v>
+      </c>
+      <c r="N11" s="11" t="n">
         <v>94</v>
       </c>
-      <c r="N11" s="11" t="n">
+      <c r="O11" s="11" t="n">
         <v>0.45</v>
       </c>
-      <c r="O11" s="11" t="n">
+      <c r="P11" s="11" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -4435,17 +4465,20 @@
         <v>3563</v>
       </c>
       <c r="J12" s="11" t="n">
-        <v>2035</v>
+        <v>953</v>
       </c>
       <c r="K12" s="11" t="n">
-        <v>5526</v>
+        <v>3915</v>
       </c>
       <c r="L12" s="11" t="n">
-        <v>46364</v>
-      </c>
-      <c r="M12" s="11" t="str"/>
+        <v>3288</v>
+      </c>
+      <c r="M12" s="11" t="n">
+        <v>46958</v>
+      </c>
       <c r="N12" s="11" t="str"/>
       <c r="O12" s="11" t="str"/>
+      <c r="P12" s="11" t="str"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: Ban Mong - 16.912 tam pin theo bang Revit CT-BP, vat tu be pin, hop 40x60 gia cuong tai neo tren 6 ban ve khung
- So tam pin tung be theo bang cac to CT-BP-01..06 (BO TRI BE PIN HO BAN MONG.pdf, 30/10): 16.912 tam; store v22.
  Tinh lai catalogue, thuyet minh, bang tinh, ban ve neo, thong ke neo, vat tu neo: BE 6 152,1 kN PES-48.
- Hop 40x60 gia cuong tai neo ve tren 6 to khung CT-KC-BE (buildHuoiVanhRaftReinforcement.py --lake=ban-mong,
  goc xoay bam truc khung): 315 cum, 599 thanh, 8.911 m; DWG khung co gia cuong + so do GC-01.
- Bang thong ke vat tu be pin 6 be (buildBanMongRaftBOQ.py): tam pin / phao / inverter / phao do cap theo bang Revit,
  C52 va hop do tren CAD khop bang to khung.
- Dinh kem web muc 1-20 cung thu tu Huoi Vanh.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/docs_ban_mong/HOBANMONG_THONG_KE_VAT_TU_NEO.xlsx
+++ b/public/docs_ban_mong/HOBANMONG_THONG_KE_VAT_TU_NEO.xlsx
@@ -1828,13 +1828,13 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Cáp chính dây bờ PES-40</t>
+          <t>Cáp chính dây bờ PES-48</t>
         </is>
       </c>
       <c r="C9" s="6" t="n"/>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Polyester PES-40, MBL 475 kN, bện 8–12 tao, chống UV</t>
+          <t>Polyester PES-48, MBL undefined kN, bện 8–12 tao, chống UV</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
@@ -1939,13 +1939,13 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Cáp chính dây đáy PES-40</t>
+          <t>Cáp chính dây đáy PES-48</t>
         </is>
       </c>
       <c r="C12" s="6" t="n"/>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Polyester PES-40, MBL 475 kN</t>
+          <t>Polyester PES-48, MBL undefined kN</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
@@ -2297,7 +2297,7 @@
       <c r="C22" s="6" t="n"/>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>SS400 t = 25, rộng 200, lỗ chốt Ø32 / Ø36 (= chốt ma-nê + 4 mm); tim chốt cách mặt đất 100 mm; hàn góc 10 mm hai phía</t>
+          <t>SS400 t = 25, rộng 200, lỗ chốt Ø32 / Ø36 / Ø39 (= chốt ma-nê + 4 mm); tim chốt cách mặt đất 100 mm; hàn góc 10 mm hai phía</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
@@ -2318,7 +2318,7 @@
       </c>
       <c r="I22" s="7" t="inlineStr">
         <is>
-          <t>1 cái mỗi điểm neo, chịu cả T của dây (tới 150,4 kN); ma-nê 8.5 / 9.5 t</t>
+          <t>1 cái mỗi điểm neo, chịu cả T của dây (tới 152,1 kN); ma-nê 8.5 / 9.5 / 12 t</t>
         </is>
       </c>
     </row>
@@ -2390,7 +2390,7 @@
       <c r="C25" s="6" t="n"/>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>C25/30 chống thấm; 10 đế 2,50 m, 1 đế 2,75 m, 5 đế 3,00 m, 6 đế 3,25 m, 3 đế 3,50 m, 2 đế 3,75 m, 6 đế 4,00 m, 1 đế 4,75 m, 1 đế 5,25 m; dày 0,4 / 0,5 / 0,6 m</t>
+          <t>C25/30 chống thấm; 10 đế 2,50 m, 1 đế 2,75 m, 6 đế 3,00 m, 5 đế 3,25 m, 3 đế 3,50 m, 1 đế 3,75 m, 6 đế 4,00 m, 1 đế 4,25 m, 1 đế 4,75 m, 1 đế 5,25 m; dày 0,4 / 0,5 / 0,6 m</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
@@ -2399,7 +2399,7 @@
         </is>
       </c>
       <c r="F25" s="8" t="n">
-        <v>173.3</v>
+        <v>173.6</v>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
@@ -2407,7 +2407,7 @@
         </is>
       </c>
       <c r="H25" s="8" t="n">
-        <v>178.5</v>
+        <v>178.8</v>
       </c>
       <c r="I25" s="7" t="inlineStr">
         <is>
@@ -2436,7 +2436,7 @@
         </is>
       </c>
       <c r="F26" s="9" t="n">
-        <v>7249</v>
+        <v>7292</v>
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
@@ -2444,7 +2444,7 @@
         </is>
       </c>
       <c r="H26" s="9" t="n">
-        <v>7467</v>
+        <v>7511</v>
       </c>
       <c r="I26" s="7" t="inlineStr">
         <is>
@@ -3323,7 +3323,7 @@
       </c>
       <c r="I51" s="7" t="inlineStr">
         <is>
-          <t>Yêu cầu của mô hình cân bằng (mooringEquilibrium.ts): dây luôn vừa căng ở mọi mực nước. Đối trọng treo một mình KHÔNG giữ được bè: nếu không khóa, bè trôi 4,3–6,7 m hết hành trình dư rồi lực dây vọt tới 91–359 kN</t>
+          <t>Yêu cầu của mô hình cân bằng (mooringEquilibrium.ts): dây luôn vừa căng ở mọi mực nước. Đối trọng treo một mình KHÔNG giữ được bè: nếu không khóa, bè trôi 4,3–6,7 m hết hành trình dư rồi lực dây vọt tới 89–379 kN</t>
         </is>
       </c>
     </row>
@@ -3343,7 +3343,7 @@
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>Khóa cáp khi gió vượt ngưỡng, giữ tới lực đứt của cáp chính (PES-32: 305 kN; PES-36: 385 kN; PES-40: 475 kN) để khóa không yếu hơn cáp; mất điện / mất tín hiệu thì tự khóa (lò xo ép phanh)</t>
+          <t>Khóa cáp khi gió vượt ngưỡng, giữ tới lực đứt của cáp chính (PES-32: 305 kN; PES-36: 385 kN; PES-48: undefined kN) để khóa không yếu hơn cáp; mất điện / mất tín hiệu thì tự khóa (lò xo ép phanh)</t>
         </is>
       </c>
       <c r="E52" s="6" t="inlineStr">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="I52" s="7" t="inlineStr">
         <is>
-          <t>Lực dây, đế, cọc của bảng này chỉ đúng khi khóa làm việc. Cần: tín hiệu gió + dự phòng, kiểm tra định kỳ, thử tải; khóa hỏng thì hệ số an toàn cáp chỉ còn 1,3–3,4 (xem cảnh báo ở Header). Pre-FS gợi ý phao chỉ hướng ~2,5 t — chưa đánh giá</t>
+          <t>Lực dây, đế, cọc của bảng này chỉ đúng khi khóa làm việc. Cần: tín hiệu gió + dự phòng, kiểm tra định kỳ, thử tải; khóa hỏng thì hệ số an toàn cáp chỉ còn NaN–NaN (xem cảnh báo ở Header). Pre-FS gợi ý phao chỉ hướng ~2,5 t — chưa đánh giá</t>
         </is>
       </c>
     </row>
@@ -3519,7 +3519,7 @@
         </is>
       </c>
       <c r="F57" s="9" t="n">
-        <v>7249</v>
+        <v>7292</v>
       </c>
       <c r="G57" s="6" t="inlineStr">
         <is>
@@ -3527,7 +3527,7 @@
         </is>
       </c>
       <c r="H57" s="9" t="n">
-        <v>7467</v>
+        <v>7511</v>
       </c>
       <c r="I57" s="7" t="inlineStr">
         <is>
@@ -3634,7 +3634,7 @@
         </is>
       </c>
       <c r="F60" s="9" t="n">
-        <v>1592</v>
+        <v>1593</v>
       </c>
       <c r="G60" s="6" t="inlineStr">
         <is>
@@ -3642,7 +3642,7 @@
         </is>
       </c>
       <c r="H60" s="9" t="n">
-        <v>1640</v>
+        <v>1641</v>
       </c>
       <c r="I60" s="7" t="inlineStr">
         <is>
@@ -3675,7 +3675,7 @@
         </is>
       </c>
       <c r="F61" s="9" t="n">
-        <v>59725</v>
+        <v>59769</v>
       </c>
       <c r="G61" s="6" t="inlineStr">
         <is>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="H61" s="9" t="n">
-        <v>61834</v>
+        <v>61879</v>
       </c>
       <c r="I61" s="7" t="inlineStr">
         <is>
@@ -3861,7 +3861,7 @@
         </is>
       </c>
       <c r="C7" s="11" t="n">
-        <v>7249</v>
+        <v>7292</v>
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
@@ -3869,7 +3869,7 @@
         </is>
       </c>
       <c r="E7" s="11" t="n">
-        <v>7467</v>
+        <v>7511</v>
       </c>
       <c r="F7" s="11" t="inlineStr">
         <is>
@@ -3945,7 +3945,7 @@
         </is>
       </c>
       <c r="C10" s="11" t="n">
-        <v>1592</v>
+        <v>1593</v>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
@@ -3953,7 +3953,7 @@
         </is>
       </c>
       <c r="E10" s="11" t="n">
-        <v>1640</v>
+        <v>1641</v>
       </c>
       <c r="F10" s="11" t="inlineStr">
         <is>
@@ -3969,11 +3969,11 @@
       </c>
       <c r="B11" s="11" t="str"/>
       <c r="C11" s="11" t="n">
-        <v>59725</v>
+        <v>59769</v>
       </c>
       <c r="D11" s="11" t="str"/>
       <c r="E11" s="11" t="n">
-        <v>61834</v>
+        <v>61879</v>
       </c>
       <c r="F11" s="11" t="str"/>
     </row>
@@ -4156,7 +4156,7 @@
         <v>0.74</v>
       </c>
       <c r="P4" s="11" t="n">
-        <v>0.86</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="5">
@@ -4204,7 +4204,7 @@
         <v>10013</v>
       </c>
       <c r="N5" s="11" t="n">
-        <v>81.09999999999999</v>
+        <v>81.3</v>
       </c>
       <c r="O5" s="11" t="n">
         <v>0.7</v>
@@ -4258,13 +4258,13 @@
         <v>3663</v>
       </c>
       <c r="N6" s="11" t="n">
-        <v>77.59999999999999</v>
+        <v>76.5</v>
       </c>
       <c r="O6" s="11" t="n">
-        <v>0.67</v>
+        <v>0.66</v>
       </c>
       <c r="P6" s="11" t="n">
-        <v>0.93</v>
+        <v>0.91</v>
       </c>
     </row>
     <row r="7">
@@ -4312,13 +4312,13 @@
         <v>5373</v>
       </c>
       <c r="N7" s="11" t="n">
-        <v>82.59999999999999</v>
+        <v>82.8</v>
       </c>
       <c r="O7" s="11" t="n">
         <v>0.71</v>
       </c>
       <c r="P7" s="11" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="8">
@@ -4366,13 +4366,13 @@
         <v>6594</v>
       </c>
       <c r="N8" s="11" t="n">
-        <v>106.2</v>
+        <v>105.9</v>
       </c>
       <c r="O8" s="11" t="n">
-        <v>0.67</v>
+        <v>0.66</v>
       </c>
       <c r="P8" s="11" t="n">
-        <v>0.93</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="9">
@@ -4420,13 +4420,13 @@
         <v>10989</v>
       </c>
       <c r="N9" s="11" t="n">
-        <v>150.4</v>
+        <v>152.1</v>
       </c>
       <c r="O9" s="11" t="n">
-        <v>0.64</v>
+        <v>0.65</v>
       </c>
       <c r="P9" s="11" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="10">
@@ -12679,7 +12679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M50"/>
+  <dimension ref="A1:M51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10.83203125" customWidth="1" min="1" max="1"/>
@@ -13386,7 +13386,7 @@
         <v>24.46</v>
       </c>
       <c r="M16" s="11" t="n">
-        <v>0.98</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="17">
@@ -13433,7 +13433,7 @@
         <v>20.39</v>
       </c>
       <c r="M17" s="11" t="n">
-        <v>0.98</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="18">
@@ -13621,7 +13621,7 @@
         <v>20.39</v>
       </c>
       <c r="M21" s="11" t="n">
-        <v>0.99</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="22">
@@ -13762,7 +13762,7 @@
         <v>6.37</v>
       </c>
       <c r="M24" s="11" t="n">
-        <v>0.82</v>
+        <v>0.8100000000000001</v>
       </c>
     </row>
     <row r="25">
@@ -13832,31 +13832,31 @@
         </is>
       </c>
       <c r="E26" s="11" t="n">
-        <v>3.25</v>
+        <v>3</v>
       </c>
       <c r="F26" s="11" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="G26" s="11" t="n">
-        <v>5.26</v>
+        <v>5.37</v>
       </c>
       <c r="H26" s="11" t="n">
-        <v>201.5</v>
+        <v>164.9</v>
       </c>
       <c r="I26" s="11" t="n">
         <v>4</v>
       </c>
       <c r="J26" s="11" t="n">
-        <v>15.2</v>
+        <v>15.6</v>
       </c>
       <c r="K26" s="11" t="n">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="L26" s="11" t="n">
-        <v>13.46</v>
+        <v>13.76</v>
       </c>
       <c r="M26" s="11" t="n">
-        <v>1</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="27">
@@ -14232,7 +14232,7 @@
         <v>35.12</v>
       </c>
       <c r="M34" s="11" t="n">
-        <v>0.98</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="35">
@@ -14279,7 +14279,7 @@
         <v>16.31</v>
       </c>
       <c r="M35" s="11" t="n">
-        <v>0.97</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="36">
@@ -14302,31 +14302,31 @@
         </is>
       </c>
       <c r="E36" s="11" t="n">
-        <v>3.75</v>
+        <v>4.25</v>
       </c>
       <c r="F36" s="11" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="G36" s="11" t="n">
-        <v>7.01</v>
+        <v>7.21</v>
       </c>
       <c r="H36" s="11" t="n">
-        <v>259.4</v>
+        <v>339.2</v>
       </c>
       <c r="I36" s="11" t="n">
         <v>4</v>
       </c>
       <c r="J36" s="11" t="n">
-        <v>15.2</v>
+        <v>14.8</v>
       </c>
       <c r="K36" s="11" t="n">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="L36" s="11" t="n">
-        <v>17.92</v>
+        <v>18.41</v>
       </c>
       <c r="M36" s="11" t="n">
-        <v>0.99</v>
+        <v>0.93</v>
       </c>
     </row>
     <row r="37">
@@ -14373,7 +14373,7 @@
         <v>7.71</v>
       </c>
       <c r="M37" s="11" t="n">
-        <v>0.87</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="38">
@@ -14420,7 +14420,7 @@
         <v>16.31</v>
       </c>
       <c r="M38" s="11" t="n">
-        <v>0.97</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="39">
@@ -14439,10 +14439,10 @@
       <c r="E39" s="11" t="str"/>
       <c r="F39" s="11" t="str"/>
       <c r="G39" s="11" t="n">
-        <v>173.27</v>
+        <v>173.58</v>
       </c>
       <c r="H39" s="11" t="n">
-        <v>7249</v>
+        <v>7292</v>
       </c>
       <c r="I39" s="11" t="n">
         <v>140</v>
@@ -14571,7 +14571,7 @@
       <c r="B44" s="11" t="str"/>
       <c r="C44" s="11" t="str"/>
       <c r="D44" s="11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E44" s="11" t="n">
         <v>3</v>
@@ -14580,13 +14580,13 @@
         <v>0.4</v>
       </c>
       <c r="G44" s="11" t="n">
-        <v>18.8</v>
+        <v>24.18</v>
       </c>
       <c r="H44" s="11" t="n">
-        <v>825</v>
+        <v>989</v>
       </c>
       <c r="I44" s="11" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="J44" s="11" t="n"/>
       <c r="K44" s="11" t="n"/>
@@ -14602,7 +14602,7 @@
       <c r="B45" s="11" t="str"/>
       <c r="C45" s="11" t="str"/>
       <c r="D45" s="11" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E45" s="11" t="n">
         <v>3.25</v>
@@ -14611,13 +14611,13 @@
         <v>0.5</v>
       </c>
       <c r="G45" s="11" t="n">
-        <v>27.34</v>
+        <v>22.09</v>
       </c>
       <c r="H45" s="11" t="n">
-        <v>1209</v>
+        <v>1008</v>
       </c>
       <c r="I45" s="11" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="J45" s="11" t="n"/>
       <c r="K45" s="11" t="n"/>
@@ -14664,7 +14664,7 @@
       <c r="B47" s="11" t="str"/>
       <c r="C47" s="11" t="str"/>
       <c r="D47" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E47" s="11" t="n">
         <v>3.75</v>
@@ -14673,13 +14673,13 @@
         <v>0.5</v>
       </c>
       <c r="G47" s="11" t="n">
-        <v>14.02</v>
+        <v>7.01</v>
       </c>
       <c r="H47" s="11" t="n">
-        <v>519</v>
+        <v>259</v>
       </c>
       <c r="I47" s="11" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J47" s="11" t="n"/>
       <c r="K47" s="11" t="n"/>
@@ -14720,7 +14720,7 @@
     <row r="49">
       <c r="A49" s="11" t="inlineStr">
         <is>
-          <t>Đế 4,75 m</t>
+          <t>Đế 4,25 m</t>
         </is>
       </c>
       <c r="B49" s="11" t="str"/>
@@ -14729,16 +14729,16 @@
         <v>1</v>
       </c>
       <c r="E49" s="11" t="n">
-        <v>4.75</v>
+        <v>4.25</v>
       </c>
       <c r="F49" s="11" t="n">
         <v>0.4</v>
       </c>
       <c r="G49" s="11" t="n">
-        <v>9.01</v>
+        <v>7.21</v>
       </c>
       <c r="H49" s="11" t="n">
-        <v>413</v>
+        <v>339</v>
       </c>
       <c r="I49" s="11" t="n">
         <v>4</v>
@@ -14751,7 +14751,7 @@
     <row r="50">
       <c r="A50" s="11" t="inlineStr">
         <is>
-          <t>Đế 5,25 m</t>
+          <t>Đế 4,75 m</t>
         </is>
       </c>
       <c r="B50" s="11" t="str"/>
@@ -14760,16 +14760,16 @@
         <v>1</v>
       </c>
       <c r="E50" s="11" t="n">
-        <v>5.25</v>
+        <v>4.75</v>
       </c>
       <c r="F50" s="11" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="G50" s="11" t="n">
-        <v>13.76</v>
+        <v>9.01</v>
       </c>
       <c r="H50" s="11" t="n">
-        <v>512</v>
+        <v>413</v>
       </c>
       <c r="I50" s="11" t="n">
         <v>4</v>
@@ -14778,6 +14778,37 @@
       <c r="K50" s="11" t="n"/>
       <c r="L50" s="11" t="n"/>
       <c r="M50" s="11" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="11" t="inlineStr">
+        <is>
+          <t>Đế 5,25 m</t>
+        </is>
+      </c>
+      <c r="B51" s="11" t="str"/>
+      <c r="C51" s="11" t="str"/>
+      <c r="D51" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" s="11" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="F51" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G51" s="11" t="n">
+        <v>13.76</v>
+      </c>
+      <c r="H51" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="I51" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="J51" s="11" t="n"/>
+      <c r="K51" s="11" t="n"/>
+      <c r="L51" s="11" t="n"/>
+      <c r="M51" s="11" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -14945,7 +14976,7 @@
         </is>
       </c>
       <c r="B5" s="11" t="n">
-        <v>81.09999999999999</v>
+        <v>81.3</v>
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
@@ -14956,10 +14987,10 @@
         <v>305</v>
       </c>
       <c r="E5" s="11" t="n">
-        <v>46.8</v>
+        <v>46.9</v>
       </c>
       <c r="F5" s="11" t="n">
-        <v>56.8</v>
+        <v>56.9</v>
       </c>
       <c r="G5" s="11" t="inlineStr">
         <is>
@@ -14970,7 +15001,7 @@
         <v>172</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>3.03</v>
+        <v>3.02</v>
       </c>
       <c r="J5" s="11" t="n">
         <v>2.12</v>
@@ -14994,7 +15025,7 @@
         </is>
       </c>
       <c r="B6" s="11" t="n">
-        <v>77.59999999999999</v>
+        <v>76.5</v>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
@@ -15005,10 +15036,10 @@
         <v>305</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>44.8</v>
+        <v>44.2</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>54.3</v>
+        <v>53.6</v>
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
@@ -15019,10 +15050,10 @@
         <v>172</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>3.17</v>
+        <v>3.21</v>
       </c>
       <c r="J6" s="11" t="n">
-        <v>2.22</v>
+        <v>2.25</v>
       </c>
       <c r="K6" s="11" t="n">
         <v>9.5</v>
@@ -15043,7 +15074,7 @@
         </is>
       </c>
       <c r="B7" s="11" t="n">
-        <v>82.59999999999999</v>
+        <v>82.8</v>
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
@@ -15054,10 +15085,10 @@
         <v>305</v>
       </c>
       <c r="E7" s="11" t="n">
-        <v>47.7</v>
+        <v>47.8</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>57.8</v>
+        <v>57.9</v>
       </c>
       <c r="G7" s="11" t="inlineStr">
         <is>
@@ -15071,7 +15102,7 @@
         <v>4.06</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>2.85</v>
+        <v>2.84</v>
       </c>
       <c r="K7" s="11" t="n">
         <v>9.5</v>
@@ -15092,7 +15123,7 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>106.2</v>
+        <v>105.9</v>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
@@ -15103,10 +15134,10 @@
         <v>385</v>
       </c>
       <c r="E8" s="11" t="n">
-        <v>61.3</v>
+        <v>61.2</v>
       </c>
       <c r="F8" s="11" t="n">
-        <v>74.40000000000001</v>
+        <v>74.2</v>
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
@@ -15117,10 +15148,10 @@
         <v>235</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>3.16</v>
+        <v>3.17</v>
       </c>
       <c r="J8" s="11" t="n">
-        <v>2.21</v>
+        <v>2.22</v>
       </c>
       <c r="K8" s="11" t="n">
         <v>12</v>
@@ -15141,21 +15172,21 @@
         </is>
       </c>
       <c r="B9" s="11" t="n">
-        <v>150.4</v>
+        <v>152.1</v>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="D9" s="11" t="n">
-        <v>475</v>
+        <v>688</v>
       </c>
       <c r="E9" s="11" t="n">
-        <v>86.8</v>
+        <v>87.8</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>105.3</v>
+        <v>106.5</v>
       </c>
       <c r="G9" s="11" t="inlineStr">
         <is>
@@ -15166,10 +15197,10 @@
         <v>385</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>3.66</v>
+        <v>3.62</v>
       </c>
       <c r="J9" s="11" t="n">
-        <v>2.56</v>
+        <v>2.53</v>
       </c>
       <c r="K9" s="11" t="n">
         <v>17</v>
@@ -26176,7 +26207,7 @@
       </c>
       <c r="J197" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K197" s="11" t="inlineStr">
@@ -26231,7 +26262,7 @@
       </c>
       <c r="J198" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K198" s="11" t="inlineStr">
@@ -26286,7 +26317,7 @@
       </c>
       <c r="J199" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K199" s="11" t="inlineStr">
@@ -26341,7 +26372,7 @@
       </c>
       <c r="J200" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K200" s="11" t="inlineStr">
@@ -26396,7 +26427,7 @@
       </c>
       <c r="J201" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K201" s="11" t="inlineStr">
@@ -26451,7 +26482,7 @@
       </c>
       <c r="J202" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K202" s="11" t="inlineStr">
@@ -26510,7 +26541,7 @@
       </c>
       <c r="J203" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K203" s="11" t="inlineStr">
@@ -26565,7 +26596,7 @@
       </c>
       <c r="J204" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K204" s="11" t="inlineStr">
@@ -26620,7 +26651,7 @@
       </c>
       <c r="J205" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K205" s="11" t="inlineStr">
@@ -26675,7 +26706,7 @@
       </c>
       <c r="J206" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K206" s="11" t="inlineStr">
@@ -26730,7 +26761,7 @@
       </c>
       <c r="J207" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K207" s="11" t="inlineStr">
@@ -26785,7 +26816,7 @@
       </c>
       <c r="J208" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K208" s="11" t="inlineStr">
@@ -26840,7 +26871,7 @@
       </c>
       <c r="J209" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K209" s="11" t="inlineStr">
@@ -26899,7 +26930,7 @@
       </c>
       <c r="J210" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K210" s="11" t="inlineStr">
@@ -26954,7 +26985,7 @@
       </c>
       <c r="J211" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K211" s="11" t="inlineStr">
@@ -27009,7 +27040,7 @@
       </c>
       <c r="J212" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K212" s="11" t="inlineStr">
@@ -27064,7 +27095,7 @@
       </c>
       <c r="J213" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K213" s="11" t="inlineStr">
@@ -27119,7 +27150,7 @@
       </c>
       <c r="J214" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K214" s="11" t="inlineStr">
@@ -27174,7 +27205,7 @@
       </c>
       <c r="J215" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K215" s="11" t="inlineStr">
@@ -27229,7 +27260,7 @@
       </c>
       <c r="J216" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K216" s="11" t="inlineStr">
@@ -27284,7 +27315,7 @@
       </c>
       <c r="J217" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K217" s="11" t="inlineStr">
@@ -27339,7 +27370,7 @@
       </c>
       <c r="J218" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K218" s="11" t="inlineStr">
@@ -27394,7 +27425,7 @@
       </c>
       <c r="J219" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K219" s="11" t="inlineStr">
@@ -27449,7 +27480,7 @@
       </c>
       <c r="J220" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K220" s="11" t="inlineStr">
@@ -27504,7 +27535,7 @@
       </c>
       <c r="J221" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K221" s="11" t="inlineStr">
@@ -27563,7 +27594,7 @@
       </c>
       <c r="J222" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K222" s="11" t="inlineStr">
@@ -27618,7 +27649,7 @@
       </c>
       <c r="J223" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K223" s="11" t="inlineStr">
@@ -27673,7 +27704,7 @@
       </c>
       <c r="J224" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K224" s="11" t="inlineStr">
@@ -27728,7 +27759,7 @@
       </c>
       <c r="J225" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K225" s="11" t="inlineStr">
@@ -27783,7 +27814,7 @@
       </c>
       <c r="J226" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K226" s="11" t="inlineStr">
@@ -27838,7 +27869,7 @@
       </c>
       <c r="J227" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K227" s="11" t="inlineStr">
@@ -27893,7 +27924,7 @@
       </c>
       <c r="J228" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K228" s="11" t="inlineStr">
@@ -27948,7 +27979,7 @@
       </c>
       <c r="J229" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K229" s="11" t="inlineStr">
@@ -28003,7 +28034,7 @@
       </c>
       <c r="J230" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K230" s="11" t="inlineStr">
@@ -28058,7 +28089,7 @@
       </c>
       <c r="J231" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K231" s="11" t="inlineStr">
@@ -28113,7 +28144,7 @@
       </c>
       <c r="J232" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K232" s="11" t="inlineStr">
@@ -28168,7 +28199,7 @@
       </c>
       <c r="J233" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K233" s="11" t="inlineStr">
@@ -28223,7 +28254,7 @@
       </c>
       <c r="J234" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K234" s="11" t="inlineStr">
@@ -28278,7 +28309,7 @@
       </c>
       <c r="J235" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K235" s="11" t="inlineStr">
@@ -28333,7 +28364,7 @@
       </c>
       <c r="J236" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K236" s="11" t="inlineStr">
@@ -28388,7 +28419,7 @@
       </c>
       <c r="J237" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K237" s="11" t="inlineStr">
@@ -28443,7 +28474,7 @@
       </c>
       <c r="J238" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K238" s="11" t="inlineStr">
@@ -28498,7 +28529,7 @@
       </c>
       <c r="J239" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K239" s="11" t="inlineStr">
@@ -28553,7 +28584,7 @@
       </c>
       <c r="J240" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K240" s="11" t="inlineStr">
@@ -28612,7 +28643,7 @@
       </c>
       <c r="J241" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K241" s="11" t="inlineStr">
@@ -28667,7 +28698,7 @@
       </c>
       <c r="J242" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K242" s="11" t="inlineStr">
@@ -28726,7 +28757,7 @@
       </c>
       <c r="J243" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K243" s="11" t="inlineStr">
@@ -28781,7 +28812,7 @@
       </c>
       <c r="J244" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K244" s="11" t="inlineStr">
@@ -28836,7 +28867,7 @@
       </c>
       <c r="J245" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K245" s="11" t="inlineStr">
@@ -28891,7 +28922,7 @@
       </c>
       <c r="J246" s="11" t="inlineStr">
         <is>
-          <t>PES-40</t>
+          <t>PES-48</t>
         </is>
       </c>
       <c r="K246" s="11" t="inlineStr">
@@ -29165,7 +29196,7 @@
         <v>41</v>
       </c>
       <c r="D6" s="11" t="n">
-        <v>81.09999999999999</v>
+        <v>81.3</v>
       </c>
       <c r="E6" s="11" t="n">
         <v>0</v>
@@ -29217,7 +29248,7 @@
         <v>17</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>79.2</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="E7" s="11" t="n">
         <v>63</v>
@@ -29269,7 +29300,7 @@
         <v>15</v>
       </c>
       <c r="D8" s="11" t="n">
-        <v>77.59999999999999</v>
+        <v>76.5</v>
       </c>
       <c r="E8" s="11" t="n">
         <v>0</v>
@@ -29284,10 +29315,10 @@
         <v>600</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.93</v>
+        <v>0.92</v>
       </c>
       <c r="J8" s="11" t="n">
-        <v>0.63</v>
+        <v>0.62</v>
       </c>
       <c r="K8" s="11" t="n">
         <v>0.18</v>
@@ -29321,7 +29352,7 @@
         <v>4</v>
       </c>
       <c r="D9" s="11" t="n">
-        <v>30.4</v>
+        <v>30</v>
       </c>
       <c r="E9" s="11" t="n">
         <v>39</v>
@@ -29336,7 +29367,7 @@
         <v>350</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.37</v>
+        <v>0.36</v>
       </c>
       <c r="J9" s="11" t="n">
         <v>0.25</v>
@@ -29345,7 +29376,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="L9" s="11" t="n">
-        <v>0.24</v>
+        <v>0.23</v>
       </c>
       <c r="M9" s="11" t="n">
         <v>0.02</v>
@@ -29373,7 +29404,7 @@
         <v>22</v>
       </c>
       <c r="D10" s="11" t="n">
-        <v>82.59999999999999</v>
+        <v>82.8</v>
       </c>
       <c r="E10" s="11" t="n">
         <v>0</v>
@@ -29391,13 +29422,13 @@
         <v>0.99</v>
       </c>
       <c r="J10" s="11" t="n">
-        <v>0.67</v>
+        <v>0.68</v>
       </c>
       <c r="K10" s="11" t="n">
         <v>0.19</v>
       </c>
       <c r="L10" s="11" t="n">
-        <v>0.4</v>
+        <v>0.41</v>
       </c>
       <c r="M10" s="11" t="n">
         <v>0.08</v>
@@ -29425,7 +29456,7 @@
         <v>14</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>82.59999999999999</v>
+        <v>82.8</v>
       </c>
       <c r="E11" s="11" t="n">
         <v>56</v>
@@ -29443,7 +29474,7 @@
         <v>0.99</v>
       </c>
       <c r="J11" s="11" t="n">
-        <v>0.67</v>
+        <v>0.68</v>
       </c>
       <c r="K11" s="11" t="n">
         <v>0.19</v>
@@ -29477,7 +29508,7 @@
         <v>27</v>
       </c>
       <c r="D12" s="11" t="n">
-        <v>77.2</v>
+        <v>77</v>
       </c>
       <c r="E12" s="11" t="n">
         <v>0</v>
@@ -29492,7 +29523,7 @@
         <v>600</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.93</v>
+        <v>0.92</v>
       </c>
       <c r="J12" s="11" t="n">
         <v>0.63</v>
@@ -29529,7 +29560,7 @@
         <v>10</v>
       </c>
       <c r="D13" s="11" t="n">
-        <v>42.9</v>
+        <v>42.8</v>
       </c>
       <c r="E13" s="11" t="n">
         <v>33</v>
@@ -29581,25 +29612,25 @@
         <v>45</v>
       </c>
       <c r="D14" s="11" t="n">
-        <v>74.8</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="E14" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F14" s="11" t="n">
-        <v>8.5</v>
+        <v>12</v>
       </c>
       <c r="G14" s="11" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="H14" s="11" t="n">
         <v>600</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>0.9</v>
+        <v>0.64</v>
       </c>
       <c r="J14" s="11" t="n">
-        <v>0.61</v>
+        <v>0.49</v>
       </c>
       <c r="K14" s="11" t="n">
         <v>0.18</v>
@@ -29633,7 +29664,7 @@
         <v>5</v>
       </c>
       <c r="D15" s="11" t="n">
-        <v>113.9</v>
+        <v>114.9</v>
       </c>
       <c r="E15" s="11" t="n">
         <v>49</v>
@@ -29645,25 +29676,25 @@
         <v>39</v>
       </c>
       <c r="H15" s="11" t="n">
-        <v>450</v>
+        <v>350</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>0.97</v>
+        <v>0.98</v>
       </c>
       <c r="J15" s="11" t="n">
-        <v>0.74</v>
+        <v>0.75</v>
       </c>
       <c r="K15" s="11" t="n">
         <v>0.28</v>
       </c>
       <c r="L15" s="11" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.82</v>
       </c>
       <c r="M15" s="11" t="n">
         <v>0.24</v>
       </c>
       <c r="N15" s="11" t="n">
-        <v>0.73</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="O15" s="11" t="str"/>
       <c r="P15" s="11" t="str"/>

</xml_diff>